<commit_message>
add advance filter and vlookup
</commit_message>
<xml_diff>
--- a/marksheet and billing.xlsx
+++ b/marksheet and billing.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rohit\Excel_Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9334E28-E1F5-4758-9F3C-A6CD8EA1F22A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EA9261B-660D-40C1-9432-B62B7E2F9ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="608" activeTab="2" xr2:uid="{1477318E-431F-4BC9-AE0F-A6B1AD161D47}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="608" activeTab="1" xr2:uid="{1477318E-431F-4BC9-AE0F-A6B1AD161D47}"/>
   </bookViews>
   <sheets>
     <sheet name="marksheet" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,13 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">billing!$A$1:$K$11</definedName>
+    <definedName name="solver_eng" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_num" localSheetId="1" hidden="1">0</definedName>
+    <definedName name="solver_opt" localSheetId="1" hidden="1">billing!$M$18</definedName>
+    <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
+    <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="85">
   <si>
     <t>name of student</t>
   </si>
@@ -288,6 +295,12 @@
   </si>
   <si>
     <t>importance</t>
+  </si>
+  <si>
+    <t>discount-vlookup</t>
+  </si>
+  <si>
+    <t>before using vlookup sort values a to z</t>
   </si>
 </sst>
 </file>
@@ -439,7 +452,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -517,6 +530,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma 2" xfId="3" xr:uid="{525CE175-190E-48A4-9F1E-B1915909ABDB}"/>
@@ -856,7 +876,7 @@
       <calculatedColumnFormula>F2*G2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="9" xr3:uid="{98CDF8CF-ADCD-4DC7-8EB7-7B196CA3CEE6}" name="Discount in per%" dataDxfId="7" dataCellStyle="Percent">
-      <calculatedColumnFormula>IF(D2="wholesaler",$F$14,IF(D2="retailer",$F$15,IF(D2="consumer",$F$16)))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(D2="wholesaler",$F$13,IF(D2="retailer",$F$14,IF(D2="consumer",$F$15)))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="10" xr3:uid="{8D1040BE-8125-4AFA-AB77-4C9E5039DE06}" name="Discount in Amount" dataDxfId="6">
       <calculatedColumnFormula>H2*I2</calculatedColumnFormula>
@@ -2194,7 +2214,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A27393F6-42F2-4765-92DD-E96E400749A2}">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
@@ -2210,7 +2230,7 @@
     <col min="11" max="11" width="12.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="6" customFormat="1">
+    <row r="1" spans="1:13" s="6" customFormat="1" ht="28.8">
       <c r="A1" s="6" t="s">
         <v>32</v>
       </c>
@@ -2244,8 +2264,11 @@
       <c r="K1" s="6" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="2" spans="1:11">
+      <c r="M1" s="29" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" s="8" t="s">
         <v>41</v>
       </c>
@@ -2272,7 +2295,7 @@
         <v>100</v>
       </c>
       <c r="I2" s="26">
-        <f t="shared" ref="I2:I11" si="1">IF(D2="wholesaler",$F$14,IF(D2="retailer",$F$15,IF(D2="consumer",$F$16)))</f>
+        <f t="shared" ref="I2:I11" si="1">IF(D2="wholesaler",$F$13,IF(D2="retailer",$F$14,IF(D2="consumer",$F$15)))</f>
         <v>0.2</v>
       </c>
       <c r="J2" s="8">
@@ -2283,8 +2306,12 @@
         <f t="shared" ref="K2:K11" si="3">H2-J2</f>
         <v>80</v>
       </c>
-    </row>
-    <row r="3" spans="1:11">
+      <c r="M2" s="30">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="8" t="s">
         <v>42</v>
       </c>
@@ -2322,8 +2349,12 @@
         <f t="shared" si="3"/>
         <v>900</v>
       </c>
-    </row>
-    <row r="4" spans="1:11">
+      <c r="M3" s="30">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="8" t="s">
         <v>43</v>
       </c>
@@ -2361,8 +2392,12 @@
         <f t="shared" si="3"/>
         <v>270</v>
       </c>
-    </row>
-    <row r="5" spans="1:11">
+      <c r="M4" s="30">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" s="8" t="s">
         <v>44</v>
       </c>
@@ -2400,8 +2435,12 @@
         <f t="shared" si="3"/>
         <v>8000</v>
       </c>
-    </row>
-    <row r="6" spans="1:11">
+      <c r="M5" s="30">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" s="8" t="s">
         <v>45</v>
       </c>
@@ -2439,8 +2478,12 @@
         <f t="shared" si="3"/>
         <v>2700</v>
       </c>
-    </row>
-    <row r="7" spans="1:11">
+      <c r="M6" s="30">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7" s="8" t="s">
         <v>46</v>
       </c>
@@ -2478,8 +2521,12 @@
         <f t="shared" si="3"/>
         <v>2700</v>
       </c>
-    </row>
-    <row r="8" spans="1:11">
+      <c r="M7" s="30">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8" s="8" t="s">
         <v>47</v>
       </c>
@@ -2517,8 +2564,12 @@
         <f t="shared" si="3"/>
         <v>2240</v>
       </c>
-    </row>
-    <row r="9" spans="1:11">
+      <c r="M8" s="30">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9" s="8" t="s">
         <v>48</v>
       </c>
@@ -2556,8 +2607,12 @@
         <f t="shared" si="3"/>
         <v>2400</v>
       </c>
-    </row>
-    <row r="10" spans="1:11">
+      <c r="M9" s="30">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" s="8" t="s">
         <v>49</v>
       </c>
@@ -2595,8 +2650,12 @@
         <f t="shared" si="3"/>
         <v>900</v>
       </c>
-    </row>
-    <row r="11" spans="1:11">
+      <c r="M10" s="30">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11" s="8" t="s">
         <v>50</v>
       </c>
@@ -2634,32 +2693,72 @@
         <f t="shared" si="3"/>
         <v>8000</v>
       </c>
-    </row>
-    <row r="14" spans="1:11">
+      <c r="M11" s="30">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
+      <c r="E13" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="F13" s="9">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
       <c r="E14" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F14" s="9">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
+      <c r="E15" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="F15" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="28.2" customHeight="1">
+      <c r="H16" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="I16" s="31"/>
+    </row>
+    <row r="17" spans="8:9">
+      <c r="H17" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="I17" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="8:9">
+      <c r="H18" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="I18" s="9">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="19" spans="8:9">
+      <c r="H19" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="F14" s="9">
+      <c r="I19" s="9">
         <v>0.2</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
-      <c r="E15" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="F15" s="9">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11">
-      <c r="E16" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="F16" s="9">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="H17:I19">
+    <sortCondition ref="H18:H19"/>
+  </sortState>
+  <mergeCells count="1">
+    <mergeCell ref="H16:I16"/>
+  </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E11" xr:uid="{F726C445-45FB-47EA-86D6-5458C9588B71}">

</xml_diff>

<commit_message>
vlookup range_lookup argument true-false
</commit_message>
<xml_diff>
--- a/marksheet and billing.xlsx
+++ b/marksheet and billing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rohit\Excel_Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EA9261B-660D-40C1-9432-B62B7E2F9ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA098B1E-2CDC-4E33-B21E-ED842CAD6A68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="608" activeTab="1" xr2:uid="{1477318E-431F-4BC9-AE0F-A6B1AD161D47}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="89">
   <si>
     <t>name of student</t>
   </si>
@@ -300,7 +300,19 @@
     <t>discount-vlookup</t>
   </si>
   <si>
-    <t>before using vlookup sort values a to z</t>
+    <t>lookup table without sort</t>
+  </si>
+  <si>
+    <t>sorted lookup table</t>
+  </si>
+  <si>
+    <t>before using vlookup sort values a to z if range_lookup=True</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> range_lookup = false</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> range_lookup = true</t>
   </si>
 </sst>
 </file>
@@ -310,7 +322,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -368,6 +380,13 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -413,7 +432,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -445,6 +464,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -452,7 +480,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -524,18 +552,24 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -856,6 +890,363 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>350520</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>716280</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52C0CCC4-4960-269D-F078-A01DF85A32DB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1866900" y="3276600"/>
+          <a:ext cx="3573780" cy="2758440"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="en-IN" sz="1100" b="0" i="0">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>The VLOOKUP function has an </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>optional fourth argument: range lookup</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>. This can be either </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>TRUE</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> or </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>FALSE</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>. </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-IN" sz="1100" b="0" i="0">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="171450" indent="-171450">
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>If the range lookup argument is </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>FALSE</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, VLOOKUP will find only exact matches. </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="171450" indent="-171450">
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+          </a:pPr>
+          <a:endParaRPr lang="en-IN" sz="1100" b="0" i="0">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="171450" indent="-171450">
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>If the range lookup argument is </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>TRUE</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, or if a range lookup </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>argument is not entered</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, VLOOKUP can find approximate matches. In this case, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>the lookup table must be </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="1" i="1" u="sng">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>sorted in ascending order </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>by the first column in it</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>; otherwise VLOOKUP may not return the correct value.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="171450" indent="-171450">
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+          </a:pPr>
+          <a:endParaRPr lang="en-IN" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1205,24 +1596,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="28.2" customHeight="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-      <c r="O1" s="27"/>
-      <c r="P1" s="27"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
     </row>
     <row r="2" spans="1:16" s="4" customFormat="1" ht="39" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -2214,7 +2605,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A27393F6-42F2-4765-92DD-E96E400749A2}">
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
@@ -2228,6 +2619,7 @@
     <col min="9" max="9" width="16.44140625" style="7" customWidth="1"/>
     <col min="10" max="10" width="18.77734375" customWidth="1"/>
     <col min="11" max="11" width="12.77734375" customWidth="1"/>
+    <col min="13" max="13" width="12.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="6" customFormat="1" ht="28.8">
@@ -2264,7 +2656,7 @@
       <c r="K1" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="M1" s="29" t="s">
+      <c r="M1" s="27" t="s">
         <v>83</v>
       </c>
     </row>
@@ -2306,8 +2698,8 @@
         <f t="shared" ref="K2:K11" si="3">H2-J2</f>
         <v>80</v>
       </c>
-      <c r="M2" s="30">
-        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+      <c r="M2" s="28">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,TRUE)</f>
         <v>0.2</v>
       </c>
     </row>
@@ -2349,8 +2741,8 @@
         <f t="shared" si="3"/>
         <v>900</v>
       </c>
-      <c r="M3" s="30">
-        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+      <c r="M3" s="28">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,TRUE)</f>
         <v>0.1</v>
       </c>
     </row>
@@ -2392,8 +2784,8 @@
         <f t="shared" si="3"/>
         <v>270</v>
       </c>
-      <c r="M4" s="30">
-        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+      <c r="M4" s="28">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,TRUE)</f>
         <v>0.1</v>
       </c>
     </row>
@@ -2435,8 +2827,8 @@
         <f t="shared" si="3"/>
         <v>8000</v>
       </c>
-      <c r="M5" s="30">
-        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+      <c r="M5" s="28">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -2478,8 +2870,8 @@
         <f t="shared" si="3"/>
         <v>2700</v>
       </c>
-      <c r="M6" s="30">
-        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+      <c r="M6" s="28">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,TRUE)</f>
         <v>0.1</v>
       </c>
     </row>
@@ -2521,8 +2913,8 @@
         <f t="shared" si="3"/>
         <v>2700</v>
       </c>
-      <c r="M7" s="30">
-        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+      <c r="M7" s="28">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,TRUE)</f>
         <v>0.1</v>
       </c>
     </row>
@@ -2564,8 +2956,8 @@
         <f t="shared" si="3"/>
         <v>2240</v>
       </c>
-      <c r="M8" s="30">
-        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+      <c r="M8" s="28">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,TRUE)</f>
         <v>0.2</v>
       </c>
     </row>
@@ -2607,8 +2999,8 @@
         <f t="shared" si="3"/>
         <v>2400</v>
       </c>
-      <c r="M9" s="30">
-        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+      <c r="M9" s="28">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -2650,8 +3042,8 @@
         <f t="shared" si="3"/>
         <v>900</v>
       </c>
-      <c r="M10" s="30">
-        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+      <c r="M10" s="28">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -2693,8 +3085,8 @@
         <f t="shared" si="3"/>
         <v>8000</v>
       </c>
-      <c r="M11" s="30">
-        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,FALSE)</f>
+      <c r="M11" s="28">
+        <f>VLOOKUP(Table1[[#This Row],[Type of customer]],$H$17:$I$19,2,TRUE)</f>
         <v>0.2</v>
       </c>
     </row>
@@ -2707,6 +3099,9 @@
       </c>
     </row>
     <row r="14" spans="1:13">
+      <c r="D14" s="31" t="s">
+        <v>84</v>
+      </c>
       <c r="E14" s="8" t="s">
         <v>66</v>
       </c>
@@ -2715,6 +3110,7 @@
       </c>
     </row>
     <row r="15" spans="1:13">
+      <c r="D15" s="31"/>
       <c r="E15" s="8" t="s">
         <v>67</v>
       </c>
@@ -2723,41 +3119,150 @@
       </c>
     </row>
     <row r="16" spans="1:13" ht="28.2" customHeight="1">
-      <c r="H16" s="31" t="s">
-        <v>84</v>
-      </c>
-      <c r="I16" s="31"/>
-    </row>
-    <row r="17" spans="8:9">
+      <c r="H16" s="32" t="s">
+        <v>86</v>
+      </c>
+      <c r="I16" s="32"/>
+      <c r="K16" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="M16" s="27" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="17" spans="7:13">
       <c r="H17" s="8" t="s">
         <v>67</v>
       </c>
       <c r="I17" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="8:9">
+      <c r="K17" s="7">
+        <f>VLOOKUP(D2,$E$13:$F$15,2,FALSE)</f>
+        <v>0.2</v>
+      </c>
+      <c r="M17" s="7">
+        <f>VLOOKUP(D2,$H$17:$I$19,2,TRUE)</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="18" spans="7:13">
+      <c r="G18" s="33" t="s">
+        <v>85</v>
+      </c>
       <c r="H18" s="8" t="s">
         <v>66</v>
       </c>
       <c r="I18" s="9">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="19" spans="8:9">
+      <c r="K18" s="7">
+        <f t="shared" ref="K18:K25" si="4">VLOOKUP(D3,$E$13:$F$15,2,FALSE)</f>
+        <v>0.1</v>
+      </c>
+      <c r="M18" s="7">
+        <f t="shared" ref="M18:M26" si="5">VLOOKUP(D3,$H$17:$I$19,2,TRUE)</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="19" spans="7:13">
+      <c r="G19" s="33"/>
       <c r="H19" s="8" t="s">
         <v>65</v>
       </c>
       <c r="I19" s="9">
         <v>0.2</v>
       </c>
+      <c r="K19" s="7">
+        <f>VLOOKUP(D4,$E$13:$F$15,2,FALSE)</f>
+        <v>0.1</v>
+      </c>
+      <c r="M19" s="7">
+        <f t="shared" si="5"/>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="20" spans="7:13">
+      <c r="K20" s="7">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="M20" s="7">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="7:13">
+      <c r="K21" s="7">
+        <f t="shared" si="4"/>
+        <v>0.1</v>
+      </c>
+      <c r="M21" s="7">
+        <f t="shared" si="5"/>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="22" spans="7:13">
+      <c r="K22" s="7">
+        <f t="shared" si="4"/>
+        <v>0.1</v>
+      </c>
+      <c r="M22" s="7">
+        <f t="shared" si="5"/>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="23" spans="7:13">
+      <c r="K23" s="7">
+        <f t="shared" si="4"/>
+        <v>0.2</v>
+      </c>
+      <c r="M23" s="7">
+        <f t="shared" si="5"/>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="24" spans="7:13">
+      <c r="K24" s="7">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="M24" s="7">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="7:13">
+      <c r="K25" s="7">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="M25" s="7">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="7:13">
+      <c r="K26" s="7">
+        <f>VLOOKUP(D11,$E$13:$F$15,2,FALSE)</f>
+        <v>0.2</v>
+      </c>
+      <c r="M26" s="7">
+        <f t="shared" si="5"/>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="27" spans="7:13">
+      <c r="M27" s="7"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="H17:I19">
     <sortCondition ref="H18:H19"/>
   </sortState>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="H16:I16"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="G18:G19"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="1">
@@ -2766,8 +3271,9 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2790,14 +3296,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="28"/>
+      <c r="B1" s="30"/>
     </row>
     <row r="2" spans="1:12">
-      <c r="A2" s="28"/>
-      <c r="B2" s="28"/>
+      <c r="A2" s="30"/>
+      <c r="B2" s="30"/>
     </row>
     <row r="3" spans="1:12" ht="18.600000000000001" customHeight="1">
       <c r="A3" s="22"/>

</xml_diff>